<commit_message>
Update parliament data - 2026-10-07
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -320,6 +320,15 @@
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20264418</t>
   </si>
   <si>
+    <t xml:space="preserve">Staatspolitik|Sozialer Schutz|Gesundheit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politique d'Etat|Protection sociale|Santé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politica nazionale|Protezione sociale|Salute</t>
+  </si>
+  <si>
     <t xml:space="preserve">26.4338</t>
   </si>
   <si>
@@ -432,15 +441,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20264261</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Staatspolitik|Sozialer Schutz|Gesundheit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politique d'Etat|Protection sociale|Santé</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politica nazionale|Protezione sociale|Salute</t>
   </si>
   <si>
     <t xml:space="preserve">26.3891</t>
@@ -6370,9 +6370,15 @@
       <c r="Q7" t="s">
         <v>53</v>
       </c>
-      <c r="R7"/>
-      <c r="S7"/>
-      <c r="T7"/>
+      <c r="R7" t="s">
+        <v>102</v>
+      </c>
+      <c r="S7" t="s">
+        <v>103</v>
+      </c>
+      <c r="T7" t="s">
+        <v>104</v>
+      </c>
       <c r="U7" t="s">
         <v>97</v>
       </c>
@@ -6383,7 +6389,7 @@
         <v>20264338</v>
       </c>
       <c r="B8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C8" t="s">
         <v>42</v>
@@ -6395,7 +6401,7 @@
         <v>25</v>
       </c>
       <c r="F8" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="G8" t="s">
         <v>27</v>
@@ -6405,38 +6411,38 @@
         <v>46</v>
       </c>
       <c r="J8" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="K8" t="s">
         <v>48</v>
       </c>
       <c r="L8" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="M8"/>
       <c r="N8" t="s">
         <v>50</v>
       </c>
       <c r="O8" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="P8" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="Q8" t="s">
         <v>36</v>
       </c>
       <c r="R8" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="S8" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="T8" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="U8" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="V8"/>
     </row>
@@ -6445,7 +6451,7 @@
         <v>20264339</v>
       </c>
       <c r="B9" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C9" t="s">
         <v>58</v>
@@ -6457,7 +6463,7 @@
         <v>25</v>
       </c>
       <c r="F9" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="G9" t="s">
         <v>27</v>
@@ -6467,38 +6473,38 @@
         <v>46</v>
       </c>
       <c r="J9" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="K9" t="s">
         <v>48</v>
       </c>
       <c r="L9" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="M9"/>
       <c r="N9" t="s">
         <v>50</v>
       </c>
       <c r="O9" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="P9" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="Q9" t="s">
         <v>36</v>
       </c>
       <c r="R9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="S9" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="T9" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="U9" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="V9"/>
     </row>
@@ -6507,7 +6513,7 @@
         <v>20267901</v>
       </c>
       <c r="B10" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C10" t="s">
         <v>23</v>
@@ -6519,50 +6525,50 @@
         <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="G10" t="s">
         <v>27</v>
       </c>
       <c r="H10" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I10" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="J10" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="K10"/>
       <c r="L10" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="M10" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="N10" t="s">
         <v>33</v>
       </c>
       <c r="O10" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="P10" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="Q10" t="s">
         <v>36</v>
       </c>
       <c r="R10" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="S10" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="T10" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="U10" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="V10"/>
     </row>
@@ -6571,19 +6577,19 @@
         <v>20264261</v>
       </c>
       <c r="B11" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C11" t="s">
         <v>58</v>
       </c>
       <c r="D11" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E11" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F11" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="G11" t="s">
         <v>45</v>
@@ -6593,38 +6599,38 @@
         <v>46</v>
       </c>
       <c r="J11" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="K11" t="s">
         <v>48</v>
       </c>
       <c r="L11" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="M11"/>
       <c r="N11" t="s">
         <v>50</v>
       </c>
       <c r="O11" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="P11" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="Q11" t="s">
         <v>36</v>
       </c>
       <c r="R11" t="s">
-        <v>140</v>
+        <v>102</v>
       </c>
       <c r="S11" t="s">
-        <v>141</v>
+        <v>103</v>
       </c>
       <c r="T11" t="s">
-        <v>142</v>
+        <v>104</v>
       </c>
       <c r="U11" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="V11"/>
     </row>
@@ -6639,10 +6645,10 @@
         <v>58</v>
       </c>
       <c r="D12" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F12" t="s">
         <v>144</v>
@@ -6961,10 +6967,10 @@
         <v>42</v>
       </c>
       <c r="D17" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E17" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F17" t="s">
         <v>204</v>
@@ -7533,10 +7539,10 @@
         <v>308</v>
       </c>
       <c r="D26" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E26" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F26" t="s">
         <v>309</v>
@@ -7611,7 +7617,7 @@
         <v>27</v>
       </c>
       <c r="H27" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I27" t="s">
         <v>323</v>
@@ -7677,7 +7683,7 @@
         <v>27</v>
       </c>
       <c r="H28" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I28" t="s">
         <v>336</v>
@@ -7875,7 +7881,7 @@
         <v>27</v>
       </c>
       <c r="H31" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I31" t="s">
         <v>372</v>
@@ -7929,10 +7935,10 @@
         <v>308</v>
       </c>
       <c r="D32" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E32" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F32" t="s">
         <v>380</v>
@@ -8007,7 +8013,7 @@
         <v>27</v>
       </c>
       <c r="H33" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I33" t="s">
         <v>395</v>
@@ -8071,7 +8077,7 @@
         <v>27</v>
       </c>
       <c r="H34" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I34" t="s">
         <v>405</v>
@@ -8189,10 +8195,10 @@
         <v>58</v>
       </c>
       <c r="D36" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E36" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F36" t="s">
         <v>219</v>
@@ -8267,7 +8273,7 @@
         <v>27</v>
       </c>
       <c r="H37" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I37" t="s">
         <v>441</v>
@@ -8715,10 +8721,10 @@
         <v>42</v>
       </c>
       <c r="D44" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E44" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F44" t="s">
         <v>520</v>
@@ -8793,7 +8799,7 @@
         <v>27</v>
       </c>
       <c r="H45" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I45" t="s">
         <v>531</v>
@@ -9229,10 +9235,10 @@
         <v>42</v>
       </c>
       <c r="D52" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E52" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F52" t="s">
         <v>608</v>
@@ -9295,10 +9301,10 @@
         <v>308</v>
       </c>
       <c r="D53" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E53" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F53" t="s">
         <v>608</v>
@@ -9364,7 +9370,7 @@
         <v>631</v>
       </c>
       <c r="E54" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F54" t="s">
         <v>632</v>
@@ -9952,7 +9958,7 @@
         <v>725</v>
       </c>
       <c r="E63" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F63" t="s">
         <v>726</v>
@@ -10015,10 +10021,10 @@
         <v>58</v>
       </c>
       <c r="D64" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E64" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F64" t="s">
         <v>735</v>
@@ -10027,7 +10033,7 @@
         <v>45</v>
       </c>
       <c r="H64" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I64" t="s">
         <v>736</v>
@@ -10150,7 +10156,7 @@
         <v>759</v>
       </c>
       <c r="E66" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F66" t="s">
         <v>760</v>
@@ -10412,7 +10418,7 @@
         <v>803</v>
       </c>
       <c r="E70" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F70" t="s">
         <v>787</v>
@@ -10421,7 +10427,7 @@
         <v>27</v>
       </c>
       <c r="H70" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I70" t="s">
         <v>804</v>
@@ -10858,7 +10864,7 @@
         <v>883</v>
       </c>
       <c r="E77" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F77" t="s">
         <v>859</v>
@@ -11578,7 +11584,7 @@
         <v>1005</v>
       </c>
       <c r="E88" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F88" t="s">
         <v>1006</v>
@@ -11644,7 +11650,7 @@
         <v>1019</v>
       </c>
       <c r="E89" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F89" t="s">
         <v>1006</v>
@@ -11776,7 +11782,7 @@
         <v>1040</v>
       </c>
       <c r="E91" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F91" t="s">
         <v>1041</v>
@@ -11839,10 +11845,10 @@
         <v>42</v>
       </c>
       <c r="D92" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E92" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F92" t="s">
         <v>1041</v>
@@ -11908,7 +11914,7 @@
         <v>631</v>
       </c>
       <c r="E93" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F93" t="s">
         <v>1061</v>
@@ -12348,7 +12354,7 @@
         <v>1138</v>
       </c>
       <c r="E100" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F100" t="s">
         <v>1115</v>
@@ -12612,7 +12618,7 @@
         <v>803</v>
       </c>
       <c r="E104" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F104" t="s">
         <v>1185</v>
@@ -13242,7 +13248,7 @@
         <v>1293</v>
       </c>
       <c r="E114" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F114" t="s">
         <v>1294</v>
@@ -13251,7 +13257,7 @@
         <v>27</v>
       </c>
       <c r="H114" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I114" t="s">
         <v>1295</v>
@@ -13440,7 +13446,7 @@
         <v>1327</v>
       </c>
       <c r="E117" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F117" t="s">
         <v>1294</v>
@@ -13449,7 +13455,7 @@
         <v>27</v>
       </c>
       <c r="H117" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I117" t="s">
         <v>1328</v>
@@ -13515,7 +13521,7 @@
         <v>27</v>
       </c>
       <c r="H118" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I118" t="s">
         <v>1338</v>
@@ -13702,7 +13708,7 @@
         <v>1327</v>
       </c>
       <c r="E121" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F121" t="s">
         <v>1363</v>
@@ -14024,7 +14030,7 @@
         <v>883</v>
       </c>
       <c r="E126" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F126" t="s">
         <v>1400</v>
@@ -14284,7 +14290,7 @@
         <v>725</v>
       </c>
       <c r="E130" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F130" t="s">
         <v>1433</v>
@@ -14293,7 +14299,7 @@
         <v>27</v>
       </c>
       <c r="H130" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I130" t="s">
         <v>1442</v>
@@ -15258,7 +15264,7 @@
         <v>631</v>
       </c>
       <c r="E145" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F145" t="s">
         <v>1597</v>
@@ -15324,7 +15330,7 @@
         <v>1606</v>
       </c>
       <c r="E146" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F146" t="s">
         <v>1597</v>
@@ -15399,7 +15405,7 @@
         <v>27</v>
       </c>
       <c r="H147" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I147" t="s">
         <v>1620</v>
@@ -15522,7 +15528,7 @@
         <v>1606</v>
       </c>
       <c r="E149" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F149" t="s">
         <v>1597</v>
@@ -15654,7 +15660,7 @@
         <v>1664</v>
       </c>
       <c r="E151" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F151" t="s">
         <v>1665</v>
@@ -16383,7 +16389,7 @@
         <v>27</v>
       </c>
       <c r="H162" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I162" t="s">
         <v>1775</v>
@@ -16437,10 +16443,10 @@
         <v>58</v>
       </c>
       <c r="D163" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E163" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F163" t="s">
         <v>1783</v>
@@ -16764,7 +16770,7 @@
         <v>1606</v>
       </c>
       <c r="E168" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F168" t="s">
         <v>1831</v>
@@ -16833,7 +16839,7 @@
       </c>
       <c r="G169"/>
       <c r="H169" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I169" t="s">
         <v>1843</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-10-21
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -152,6 +152,9 @@
     <t xml:space="preserve">SR</t>
   </si>
   <si>
+    <t xml:space="preserve">UVEK</t>
+  </si>
+  <si>
     <t xml:space="preserve">Titel folgt</t>
   </si>
   <si>
@@ -194,9 +197,6 @@
     <t xml:space="preserve">2026-06-04</t>
   </si>
   <si>
-    <t xml:space="preserve">UVEK</t>
-  </si>
-  <si>
     <t xml:space="preserve">Wie sieht bei der Post die geografische Verteilung der Arbeitsplätze aus?</t>
   </si>
   <si>
@@ -371,6 +371,9 @@
     <t xml:space="preserve">26.4339</t>
   </si>
   <si>
+    <t xml:space="preserve">WBF</t>
+  </si>
+  <si>
     <t xml:space="preserve">Chômage des seniors : la Confédération se désengage-t-elle au pire moment ?</t>
   </si>
   <si>
@@ -396,9 +399,6 @@
   </si>
   <si>
     <t xml:space="preserve">2026-09-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WBF</t>
   </si>
   <si>
     <t xml:space="preserve">Mercosur: Wie sollen die 517 Millionen für die Landwirtschaft finanziert werden?</t>
@@ -6096,40 +6096,42 @@
       <c r="G3" t="s">
         <v>45</v>
       </c>
-      <c r="H3"/>
+      <c r="H3" t="s">
+        <v>46</v>
+      </c>
       <c r="I3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="K3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="L3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M3"/>
       <c r="N3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="O3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="P3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="S3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="T3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="U3" t="s">
         <v>44</v>
@@ -6141,10 +6143,10 @@
         <v>20263563</v>
       </c>
       <c r="B4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D4" t="s">
         <v>24</v>
@@ -6153,13 +6155,13 @@
         <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G4" t="s">
         <v>27</v>
       </c>
       <c r="H4" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I4" t="s">
         <v>61</v>
@@ -6210,7 +6212,7 @@
         <v>71</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
         <v>24</v>
@@ -6219,7 +6221,7 @@
         <v>25</v>
       </c>
       <c r="F5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G5" t="s">
         <v>27</v>
@@ -6285,7 +6287,7 @@
         <v>85</v>
       </c>
       <c r="F6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G6" t="s">
         <v>45</v>
@@ -6318,7 +6320,7 @@
         <v>92</v>
       </c>
       <c r="Q6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R6" t="s">
         <v>93</v>
@@ -6342,7 +6344,7 @@
         <v>96</v>
       </c>
       <c r="C7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D7" t="s">
         <v>24</v>
@@ -6356,7 +6358,9 @@
       <c r="G7" t="s">
         <v>27</v>
       </c>
-      <c r="H7"/>
+      <c r="H7" t="s">
+        <v>72</v>
+      </c>
       <c r="I7" t="s">
         <v>98</v>
       </c>
@@ -6364,7 +6368,7 @@
         <v>99</v>
       </c>
       <c r="K7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="L7" t="s">
         <v>100</v>
@@ -6373,7 +6377,7 @@
         <v>101</v>
       </c>
       <c r="N7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="O7" t="s">
         <v>102</v>
@@ -6382,7 +6386,7 @@
         <v>103</v>
       </c>
       <c r="Q7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R7" t="s">
         <v>104</v>
@@ -6420,7 +6424,9 @@
       <c r="G8" t="s">
         <v>27</v>
       </c>
-      <c r="H8"/>
+      <c r="H8" t="s">
+        <v>72</v>
+      </c>
       <c r="I8" t="s">
         <v>109</v>
       </c>
@@ -6428,7 +6434,7 @@
         <v>110</v>
       </c>
       <c r="K8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="L8" t="s">
         <v>111</v>
@@ -6437,7 +6443,7 @@
         <v>112</v>
       </c>
       <c r="N8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="O8" t="s">
         <v>113</v>
@@ -6470,7 +6476,7 @@
         <v>118</v>
       </c>
       <c r="C9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D9" t="s">
         <v>24</v>
@@ -6484,40 +6490,42 @@
       <c r="G9" t="s">
         <v>27</v>
       </c>
-      <c r="H9"/>
+      <c r="H9" t="s">
+        <v>119</v>
+      </c>
       <c r="I9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="L9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="M9"/>
       <c r="N9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="O9" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="Q9" t="s">
         <v>36</v>
       </c>
       <c r="R9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="S9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="T9" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="U9" t="s">
         <v>108</v>
@@ -6529,7 +6537,7 @@
         <v>20267901</v>
       </c>
       <c r="B10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C10" t="s">
         <v>23</v>
@@ -6541,13 +6549,13 @@
         <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G10" t="s">
         <v>27</v>
       </c>
       <c r="H10" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I10" t="s">
         <v>129</v>
@@ -6596,7 +6604,7 @@
         <v>139</v>
       </c>
       <c r="C11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D11" t="s">
         <v>140</v>
@@ -6610,22 +6618,24 @@
       <c r="G11" t="s">
         <v>45</v>
       </c>
-      <c r="H11"/>
+      <c r="H11" t="s">
+        <v>72</v>
+      </c>
       <c r="I11" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J11" t="s">
         <v>143</v>
       </c>
       <c r="K11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="L11" t="s">
         <v>144</v>
       </c>
       <c r="M11"/>
       <c r="N11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="O11" t="s">
         <v>145</v>
@@ -6658,7 +6668,7 @@
         <v>147</v>
       </c>
       <c r="C12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D12" t="s">
         <v>140</v>
@@ -6869,7 +6879,7 @@
         <v>27</v>
       </c>
       <c r="H15" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I15" t="s">
         <v>189</v>
@@ -6932,22 +6942,24 @@
       <c r="G16" t="s">
         <v>27</v>
       </c>
-      <c r="H16"/>
+      <c r="H16" t="s">
+        <v>72</v>
+      </c>
       <c r="I16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J16" t="s">
         <v>200</v>
       </c>
       <c r="K16" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="L16" t="s">
         <v>201</v>
       </c>
       <c r="M16"/>
       <c r="N16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="O16" t="s">
         <v>202</v>
@@ -7086,7 +7098,7 @@
         <v>228</v>
       </c>
       <c r="Q18" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R18" t="s">
         <v>93</v>
@@ -7110,7 +7122,7 @@
         <v>229</v>
       </c>
       <c r="C19" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D19" t="s">
         <v>230</v>
@@ -7124,22 +7136,24 @@
       <c r="G19" t="s">
         <v>27</v>
       </c>
-      <c r="H19"/>
+      <c r="H19" t="s">
+        <v>46</v>
+      </c>
       <c r="I19" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J19" t="s">
         <v>232</v>
       </c>
       <c r="K19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="L19" t="s">
         <v>233</v>
       </c>
       <c r="M19"/>
       <c r="N19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="O19" t="s">
         <v>234</v>
@@ -7187,7 +7201,7 @@
         <v>27</v>
       </c>
       <c r="H20" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I20" t="s">
         <v>240</v>
@@ -7236,7 +7250,7 @@
         <v>249</v>
       </c>
       <c r="C21" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D21" t="s">
         <v>250</v>
@@ -7250,7 +7264,9 @@
       <c r="G21" t="s">
         <v>27</v>
       </c>
-      <c r="H21"/>
+      <c r="H21" t="s">
+        <v>28</v>
+      </c>
       <c r="I21" t="s">
         <v>251</v>
       </c>
@@ -7265,7 +7281,7 @@
         <v>254</v>
       </c>
       <c r="N21" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="O21" t="s">
         <v>255</v>
@@ -7274,7 +7290,7 @@
         <v>256</v>
       </c>
       <c r="Q21" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R21" t="s">
         <v>257</v>
@@ -7336,7 +7352,7 @@
         <v>272</v>
       </c>
       <c r="Q22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R22"/>
       <c r="S22"/>
@@ -7354,7 +7370,7 @@
         <v>274</v>
       </c>
       <c r="C23" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D23" t="s">
         <v>43</v>
@@ -7369,7 +7385,7 @@
         <v>45</v>
       </c>
       <c r="H23" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I23" t="s">
         <v>275</v>
@@ -7420,7 +7436,7 @@
         <v>287</v>
       </c>
       <c r="C24" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D24" t="s">
         <v>288</v>
@@ -7435,7 +7451,7 @@
         <v>27</v>
       </c>
       <c r="H24" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I24" t="s">
         <v>290</v>
@@ -7486,7 +7502,7 @@
         <v>298</v>
       </c>
       <c r="C25" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D25" t="s">
         <v>299</v>
@@ -7618,7 +7634,7 @@
         <v>325</v>
       </c>
       <c r="C27" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D27" t="s">
         <v>326</v>
@@ -7633,7 +7649,7 @@
         <v>27</v>
       </c>
       <c r="H27" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I27" t="s">
         <v>327</v>
@@ -7684,7 +7700,7 @@
         <v>339</v>
       </c>
       <c r="C28" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D28" t="s">
         <v>326</v>
@@ -7699,7 +7715,7 @@
         <v>27</v>
       </c>
       <c r="H28" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I28" t="s">
         <v>340</v>
@@ -7750,7 +7766,7 @@
         <v>347</v>
       </c>
       <c r="C29" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D29" t="s">
         <v>348</v>
@@ -7765,7 +7781,7 @@
         <v>27</v>
       </c>
       <c r="H29" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I29" t="s">
         <v>350</v>
@@ -7882,7 +7898,7 @@
         <v>374</v>
       </c>
       <c r="C31" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D31" t="s">
         <v>326</v>
@@ -7897,7 +7913,7 @@
         <v>27</v>
       </c>
       <c r="H31" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I31" t="s">
         <v>376</v>
@@ -8029,7 +8045,7 @@
         <v>27</v>
       </c>
       <c r="H33" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I33" t="s">
         <v>399</v>
@@ -8093,7 +8109,7 @@
         <v>27</v>
       </c>
       <c r="H34" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I34" t="s">
         <v>409</v>
@@ -8142,7 +8158,7 @@
         <v>418</v>
       </c>
       <c r="C35" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D35" t="s">
         <v>419</v>
@@ -8208,7 +8224,7 @@
         <v>432</v>
       </c>
       <c r="C36" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D36" t="s">
         <v>140</v>
@@ -8223,7 +8239,7 @@
         <v>45</v>
       </c>
       <c r="H36" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I36" t="s">
         <v>433</v>
@@ -8289,7 +8305,7 @@
         <v>27</v>
       </c>
       <c r="H37" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I37" t="s">
         <v>445</v>
@@ -8340,7 +8356,7 @@
         <v>456</v>
       </c>
       <c r="C38" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D38" t="s">
         <v>457</v>
@@ -8355,7 +8371,7 @@
         <v>27</v>
       </c>
       <c r="H38" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I38" t="s">
         <v>458</v>
@@ -8470,7 +8486,7 @@
         <v>478</v>
       </c>
       <c r="C40" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D40" t="s">
         <v>230</v>
@@ -8485,7 +8501,7 @@
         <v>27</v>
       </c>
       <c r="H40" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I40" t="s">
         <v>479</v>
@@ -8536,7 +8552,7 @@
         <v>486</v>
       </c>
       <c r="C41" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D41" t="s">
         <v>487</v>
@@ -8644,7 +8660,7 @@
         <v>508</v>
       </c>
       <c r="Q42" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R42" t="s">
         <v>509</v>
@@ -8668,7 +8684,7 @@
         <v>513</v>
       </c>
       <c r="C43" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D43" t="s">
         <v>514</v>
@@ -8683,7 +8699,7 @@
         <v>27</v>
       </c>
       <c r="H43" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I43" t="s">
         <v>516</v>
@@ -8815,7 +8831,7 @@
         <v>27</v>
       </c>
       <c r="H45" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I45" t="s">
         <v>535</v>
@@ -9026,7 +9042,7 @@
         <v>572</v>
       </c>
       <c r="Q48" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R48" t="s">
         <v>573</v>
@@ -9092,7 +9108,7 @@
         <v>585</v>
       </c>
       <c r="Q49" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R49" t="s">
         <v>157</v>
@@ -9116,7 +9132,7 @@
         <v>586</v>
       </c>
       <c r="C50" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D50" t="s">
         <v>587</v>
@@ -9182,7 +9198,7 @@
         <v>599</v>
       </c>
       <c r="C51" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D51" t="s">
         <v>600</v>
@@ -9197,7 +9213,7 @@
         <v>27</v>
       </c>
       <c r="H51" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I51" t="s">
         <v>601</v>
@@ -9380,7 +9396,7 @@
         <v>634</v>
       </c>
       <c r="C54" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D54" t="s">
         <v>635</v>
@@ -9552,7 +9568,7 @@
         <v>663</v>
       </c>
       <c r="Q56" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R56" t="s">
         <v>664</v>
@@ -9616,7 +9632,7 @@
         <v>673</v>
       </c>
       <c r="Q57" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R57" t="s">
         <v>93</v>
@@ -9680,7 +9696,7 @@
         <v>683</v>
       </c>
       <c r="Q58" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R58" t="s">
         <v>684</v>
@@ -9746,7 +9762,7 @@
         <v>696</v>
       </c>
       <c r="Q59" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R59" t="s">
         <v>697</v>
@@ -9812,7 +9828,7 @@
         <v>708</v>
       </c>
       <c r="Q60" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R60" t="s">
         <v>497</v>
@@ -9836,7 +9852,7 @@
         <v>709</v>
       </c>
       <c r="C61" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D61" t="s">
         <v>457</v>
@@ -9851,7 +9867,7 @@
         <v>27</v>
       </c>
       <c r="H61" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I61" t="s">
         <v>710</v>
@@ -9968,7 +9984,7 @@
         <v>728</v>
       </c>
       <c r="C63" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D63" t="s">
         <v>729</v>
@@ -10034,7 +10050,7 @@
         <v>738</v>
       </c>
       <c r="C64" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D64" t="s">
         <v>140</v>
@@ -10049,7 +10065,7 @@
         <v>45</v>
       </c>
       <c r="H64" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I64" t="s">
         <v>740</v>
@@ -10100,7 +10116,7 @@
         <v>750</v>
       </c>
       <c r="C65" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D65" t="s">
         <v>751</v>
@@ -10166,7 +10182,7 @@
         <v>762</v>
       </c>
       <c r="C66" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D66" t="s">
         <v>763</v>
@@ -10313,7 +10329,7 @@
         <v>27</v>
       </c>
       <c r="H68" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I68" t="s">
         <v>792</v>
@@ -10340,7 +10356,7 @@
         <v>798</v>
       </c>
       <c r="Q68" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R68" t="s">
         <v>236</v>
@@ -10443,7 +10459,7 @@
         <v>27</v>
       </c>
       <c r="H70" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I70" t="s">
         <v>808</v>
@@ -10556,7 +10572,7 @@
         <v>828</v>
       </c>
       <c r="C72" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D72" t="s">
         <v>829</v>
@@ -10598,7 +10614,7 @@
         <v>837</v>
       </c>
       <c r="Q72" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R72" t="s">
         <v>838</v>
@@ -10662,7 +10678,7 @@
         <v>847</v>
       </c>
       <c r="Q73" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R73" t="s">
         <v>848</v>
@@ -10724,7 +10740,7 @@
         <v>860</v>
       </c>
       <c r="Q74" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R74"/>
       <c r="S74"/>
@@ -10742,7 +10758,7 @@
         <v>861</v>
       </c>
       <c r="C75" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D75" t="s">
         <v>862</v>
@@ -10757,7 +10773,7 @@
         <v>27</v>
       </c>
       <c r="H75" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I75" t="s">
         <v>864</v>
@@ -10808,7 +10824,7 @@
         <v>874</v>
       </c>
       <c r="C76" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D76" t="s">
         <v>875</v>
@@ -10823,7 +10839,7 @@
         <v>27</v>
       </c>
       <c r="H76" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I76" t="s">
         <v>876</v>
@@ -10850,7 +10866,7 @@
         <v>882</v>
       </c>
       <c r="Q76" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R76" t="s">
         <v>883</v>
@@ -10916,7 +10932,7 @@
         <v>895</v>
       </c>
       <c r="Q77" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R77" t="s">
         <v>896</v>
@@ -10983,13 +10999,13 @@
         <v>334</v>
       </c>
       <c r="R78" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="S78" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="T78" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="U78" t="s">
         <v>544</v>
@@ -11004,7 +11020,7 @@
         <v>908</v>
       </c>
       <c r="C79" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D79" t="s">
         <v>909</v>
@@ -11070,7 +11086,7 @@
         <v>920</v>
       </c>
       <c r="C80" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D80" t="s">
         <v>921</v>
@@ -11085,7 +11101,7 @@
         <v>27</v>
       </c>
       <c r="H80" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I80" t="s">
         <v>923</v>
@@ -11149,7 +11165,7 @@
         <v>27</v>
       </c>
       <c r="H81" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I81" t="s">
         <v>932</v>
@@ -11176,7 +11192,7 @@
         <v>938</v>
       </c>
       <c r="Q81" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R81" t="s">
         <v>939</v>
@@ -11200,7 +11216,7 @@
         <v>942</v>
       </c>
       <c r="C82" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D82" t="s">
         <v>701</v>
@@ -11215,7 +11231,7 @@
         <v>27</v>
       </c>
       <c r="H82" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I82" t="s">
         <v>943</v>
@@ -11266,7 +11282,7 @@
         <v>953</v>
       </c>
       <c r="C83" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D83" t="s">
         <v>954</v>
@@ -11281,7 +11297,7 @@
         <v>45</v>
       </c>
       <c r="H83" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I83" t="s">
         <v>956</v>
@@ -11308,7 +11324,7 @@
         <v>962</v>
       </c>
       <c r="Q83" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R83" t="s">
         <v>871</v>
@@ -11347,7 +11363,7 @@
         <v>27</v>
       </c>
       <c r="H84" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I84" t="s">
         <v>966</v>
@@ -11374,7 +11390,7 @@
         <v>972</v>
       </c>
       <c r="Q84" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R84" t="s">
         <v>440</v>
@@ -11636,7 +11652,7 @@
         <v>1018</v>
       </c>
       <c r="Q88" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R88" t="s">
         <v>1019</v>
@@ -11660,7 +11676,7 @@
         <v>1022</v>
       </c>
       <c r="C89" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D89" t="s">
         <v>1023</v>
@@ -11702,7 +11718,7 @@
         <v>1030</v>
       </c>
       <c r="Q89" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R89" t="s">
         <v>1031</v>
@@ -11726,7 +11742,7 @@
         <v>1034</v>
       </c>
       <c r="C90" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D90" t="s">
         <v>1035</v>
@@ -11741,7 +11757,7 @@
         <v>27</v>
       </c>
       <c r="H90" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I90" t="s">
         <v>1036</v>
@@ -11924,7 +11940,7 @@
         <v>1064</v>
       </c>
       <c r="C93" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D93" t="s">
         <v>635</v>
@@ -11939,7 +11955,7 @@
         <v>45</v>
       </c>
       <c r="H93" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I93" t="s">
         <v>1066</v>
@@ -11990,7 +12006,7 @@
         <v>1076</v>
       </c>
       <c r="C94" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D94" t="s">
         <v>909</v>
@@ -12032,7 +12048,7 @@
         <v>1084</v>
       </c>
       <c r="Q94" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R94" t="s">
         <v>1085</v>
@@ -12067,7 +12083,7 @@
       </c>
       <c r="G95"/>
       <c r="H95" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I95" t="s">
         <v>1091</v>
@@ -12094,7 +12110,7 @@
         <v>1097</v>
       </c>
       <c r="Q95" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R95"/>
       <c r="S95"/>
@@ -12150,7 +12166,7 @@
         <v>1104</v>
       </c>
       <c r="Q96" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R96"/>
       <c r="S96"/>
@@ -12208,7 +12224,7 @@
         <v>1114</v>
       </c>
       <c r="Q97" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R97" t="s">
         <v>1115</v>
@@ -12247,7 +12263,7 @@
         <v>27</v>
       </c>
       <c r="H98" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I98" t="s">
         <v>1120</v>
@@ -12274,7 +12290,7 @@
         <v>1126</v>
       </c>
       <c r="Q98" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R98" t="s">
         <v>1127</v>
@@ -12298,7 +12314,7 @@
         <v>1130</v>
       </c>
       <c r="C99" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D99" t="s">
         <v>974</v>
@@ -12364,7 +12380,7 @@
         <v>1141</v>
       </c>
       <c r="C100" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D100" t="s">
         <v>1142</v>
@@ -12562,7 +12578,7 @@
         <v>1176</v>
       </c>
       <c r="C103" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D103" t="s">
         <v>1177</v>
@@ -12643,7 +12659,7 @@
         <v>27</v>
       </c>
       <c r="H104" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I104" t="s">
         <v>1190</v>
@@ -12670,7 +12686,7 @@
         <v>1196</v>
       </c>
       <c r="Q104" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R104" t="s">
         <v>1197</v>
@@ -12694,7 +12710,7 @@
         <v>1200</v>
       </c>
       <c r="C105" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D105" t="s">
         <v>1201</v>
@@ -12709,7 +12725,7 @@
         <v>27</v>
       </c>
       <c r="H105" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I105" t="s">
         <v>1202</v>
@@ -12771,7 +12787,7 @@
       </c>
       <c r="G106"/>
       <c r="H106" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I106" t="s">
         <v>1214</v>
@@ -12798,7 +12814,7 @@
         <v>1220</v>
       </c>
       <c r="Q106" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R106"/>
       <c r="S106"/>
@@ -12858,7 +12874,7 @@
         <v>1228</v>
       </c>
       <c r="Q107" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R107" t="s">
         <v>697</v>
@@ -12922,7 +12938,7 @@
         <v>1237</v>
       </c>
       <c r="Q108" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R108" t="s">
         <v>1238</v>
@@ -12961,7 +12977,7 @@
         <v>27</v>
       </c>
       <c r="H109" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I109" t="s">
         <v>1244</v>
@@ -12986,7 +13002,7 @@
         <v>1249</v>
       </c>
       <c r="Q109" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R109" t="s">
         <v>1127</v>
@@ -13106,7 +13122,7 @@
         <v>1268</v>
       </c>
       <c r="Q111" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R111" t="s">
         <v>1269</v>
@@ -13141,7 +13157,7 @@
       </c>
       <c r="G112"/>
       <c r="H112" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I112" t="s">
         <v>1273</v>
@@ -13168,7 +13184,7 @@
         <v>1280</v>
       </c>
       <c r="Q112" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R112" t="s">
         <v>1281</v>
@@ -13273,7 +13289,7 @@
         <v>27</v>
       </c>
       <c r="H114" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I114" t="s">
         <v>1299</v>
@@ -13324,7 +13340,7 @@
         <v>1309</v>
       </c>
       <c r="C115" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D115" t="s">
         <v>1310</v>
@@ -13339,7 +13355,7 @@
         <v>27</v>
       </c>
       <c r="H115" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I115" t="s">
         <v>1311</v>
@@ -13366,7 +13382,7 @@
         <v>1317</v>
       </c>
       <c r="Q115" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R115" t="s">
         <v>950</v>
@@ -13456,7 +13472,7 @@
         <v>1330</v>
       </c>
       <c r="C117" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D117" t="s">
         <v>1331</v>
@@ -13471,7 +13487,7 @@
         <v>27</v>
       </c>
       <c r="H117" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I117" t="s">
         <v>1332</v>
@@ -13537,7 +13553,7 @@
         <v>27</v>
       </c>
       <c r="H118" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I118" t="s">
         <v>1342</v>
@@ -13652,7 +13668,7 @@
         <v>1357</v>
       </c>
       <c r="C120" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D120" t="s">
         <v>326</v>
@@ -13667,7 +13683,7 @@
         <v>27</v>
       </c>
       <c r="H120" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I120" t="s">
         <v>1359</v>
@@ -13733,7 +13749,7 @@
         <v>27</v>
       </c>
       <c r="H121" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I121" t="s">
         <v>1368</v>
@@ -13758,7 +13774,7 @@
         <v>1373</v>
       </c>
       <c r="Q121" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R121" t="s">
         <v>236</v>
@@ -13974,7 +13990,7 @@
         <v>1391</v>
       </c>
       <c r="C125" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D125" t="s">
         <v>829</v>
@@ -14016,7 +14032,7 @@
         <v>1399</v>
       </c>
       <c r="Q125" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R125" t="s">
         <v>1400</v>
@@ -14040,7 +14056,7 @@
         <v>1403</v>
       </c>
       <c r="C126" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D126" t="s">
         <v>887</v>
@@ -14082,7 +14098,7 @@
         <v>1411</v>
       </c>
       <c r="Q126" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R126" t="s">
         <v>474</v>
@@ -14106,7 +14122,7 @@
         <v>1412</v>
       </c>
       <c r="C127" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D127" t="s">
         <v>1413</v>
@@ -14121,7 +14137,7 @@
         <v>27</v>
       </c>
       <c r="H127" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I127" t="s">
         <v>1414</v>
@@ -14148,7 +14164,7 @@
         <v>1420</v>
       </c>
       <c r="Q127" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R127" t="s">
         <v>1421</v>
@@ -14172,7 +14188,7 @@
         <v>1424</v>
       </c>
       <c r="C128" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D128" t="s">
         <v>1425</v>
@@ -14276,7 +14292,7 @@
         <v>1444</v>
       </c>
       <c r="Q129" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R129" t="s">
         <v>204</v>
@@ -14315,7 +14331,7 @@
         <v>27</v>
       </c>
       <c r="H130" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I130" t="s">
         <v>1446</v>
@@ -14432,7 +14448,7 @@
         <v>1468</v>
       </c>
       <c r="C132" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D132" t="s">
         <v>1469</v>
@@ -14513,7 +14529,7 @@
         <v>27</v>
       </c>
       <c r="H133" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I133" t="s">
         <v>1478</v>
@@ -14606,7 +14622,7 @@
         <v>1496</v>
       </c>
       <c r="Q134" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R134" t="s">
         <v>1497</v>
@@ -14630,7 +14646,7 @@
         <v>1500</v>
       </c>
       <c r="C135" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D135" t="s">
         <v>230</v>
@@ -14645,7 +14661,7 @@
         <v>27</v>
       </c>
       <c r="H135" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I135" t="s">
         <v>1502</v>
@@ -14672,7 +14688,7 @@
         <v>1508</v>
       </c>
       <c r="Q135" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R135" t="s">
         <v>195</v>
@@ -14802,7 +14818,7 @@
         <v>1526</v>
       </c>
       <c r="Q137" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R137" t="s">
         <v>995</v>
@@ -14841,7 +14857,7 @@
         <v>27</v>
       </c>
       <c r="H138" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I138" t="s">
         <v>1529</v>
@@ -14866,7 +14882,7 @@
         <v>1534</v>
       </c>
       <c r="Q138" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R138" t="s">
         <v>246</v>
@@ -14905,7 +14921,7 @@
         <v>27</v>
       </c>
       <c r="H139" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I139" t="s">
         <v>1537</v>
@@ -15052,7 +15068,7 @@
         <v>1562</v>
       </c>
       <c r="Q141" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R141" t="s">
         <v>1563</v>
@@ -15076,7 +15092,7 @@
         <v>1566</v>
       </c>
       <c r="C142" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D142" t="s">
         <v>1567</v>
@@ -15091,7 +15107,7 @@
         <v>27</v>
       </c>
       <c r="H142" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I142" t="s">
         <v>1569</v>
@@ -15142,7 +15158,7 @@
         <v>1579</v>
       </c>
       <c r="C143" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D143" t="s">
         <v>1580</v>
@@ -15208,7 +15224,7 @@
         <v>1592</v>
       </c>
       <c r="C144" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D144" t="s">
         <v>43</v>
@@ -15223,7 +15239,7 @@
         <v>45</v>
       </c>
       <c r="H144" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I144" t="s">
         <v>1593</v>
@@ -15250,7 +15266,7 @@
         <v>1599</v>
       </c>
       <c r="Q144" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R144" t="s">
         <v>950</v>
@@ -15355,7 +15371,7 @@
         <v>27</v>
       </c>
       <c r="H146" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I146" t="s">
         <v>1611</v>
@@ -15421,7 +15437,7 @@
         <v>27</v>
       </c>
       <c r="H147" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I147" t="s">
         <v>1624</v>
@@ -15472,7 +15488,7 @@
         <v>1634</v>
       </c>
       <c r="C148" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D148" t="s">
         <v>600</v>
@@ -15487,7 +15503,7 @@
         <v>27</v>
       </c>
       <c r="H148" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I148" t="s">
         <v>1635</v>
@@ -15514,7 +15530,7 @@
         <v>1641</v>
       </c>
       <c r="Q148" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R148" t="s">
         <v>1642</v>
@@ -15538,7 +15554,7 @@
         <v>1645</v>
       </c>
       <c r="C149" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D149" t="s">
         <v>1610</v>
@@ -15580,7 +15596,7 @@
         <v>1652</v>
       </c>
       <c r="Q149" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R149" t="s">
         <v>1653</v>
@@ -15604,7 +15620,7 @@
         <v>1656</v>
       </c>
       <c r="C150" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D150" t="s">
         <v>1319</v>
@@ -15670,7 +15686,7 @@
         <v>1667</v>
       </c>
       <c r="C151" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D151" t="s">
         <v>1668</v>
@@ -15736,7 +15752,7 @@
         <v>1677</v>
       </c>
       <c r="C152" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D152" t="s">
         <v>501</v>
@@ -15778,7 +15794,7 @@
         <v>1685</v>
       </c>
       <c r="Q152" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R152" t="s">
         <v>596</v>
@@ -15802,7 +15818,7 @@
         <v>1686</v>
       </c>
       <c r="C153" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D153" t="s">
         <v>1687</v>
@@ -15844,7 +15860,7 @@
         <v>1695</v>
       </c>
       <c r="Q153" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R153" t="s">
         <v>917</v>
@@ -15910,7 +15926,7 @@
         <v>1705</v>
       </c>
       <c r="Q154" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R154" t="s">
         <v>1465</v>
@@ -15949,7 +15965,7 @@
         <v>27</v>
       </c>
       <c r="H155" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I155" t="s">
         <v>1707</v>
@@ -16013,7 +16029,7 @@
         <v>27</v>
       </c>
       <c r="H156" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I156" t="s">
         <v>1715</v>
@@ -16038,7 +16054,7 @@
         <v>1720</v>
       </c>
       <c r="Q156" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R156" t="s">
         <v>195</v>
@@ -16126,7 +16142,7 @@
         <v>1734</v>
       </c>
       <c r="C158" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D158" t="s">
         <v>1035</v>
@@ -16141,7 +16157,7 @@
         <v>27</v>
       </c>
       <c r="H158" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I158" t="s">
         <v>1736</v>
@@ -16390,7 +16406,7 @@
         <v>1776</v>
       </c>
       <c r="C162" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D162" t="s">
         <v>1777</v>
@@ -16405,7 +16421,7 @@
         <v>27</v>
       </c>
       <c r="H162" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I162" t="s">
         <v>1779</v>
@@ -16456,7 +16472,7 @@
         <v>1786</v>
       </c>
       <c r="C163" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D163" t="s">
         <v>140</v>
@@ -16471,7 +16487,7 @@
         <v>45</v>
       </c>
       <c r="H163" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I163" t="s">
         <v>1788</v>
@@ -16498,7 +16514,7 @@
         <v>1794</v>
       </c>
       <c r="Q163" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R163" t="s">
         <v>1795</v>
@@ -16522,7 +16538,7 @@
         <v>1798</v>
       </c>
       <c r="C164" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D164" t="s">
         <v>829</v>
@@ -16537,7 +16553,7 @@
         <v>27</v>
       </c>
       <c r="H164" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I164" t="s">
         <v>1800</v>
@@ -16564,7 +16580,7 @@
         <v>1806</v>
       </c>
       <c r="Q164" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R164" t="s">
         <v>1807</v>
@@ -16603,7 +16619,7 @@
         <v>27</v>
       </c>
       <c r="H165" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I165" t="s">
         <v>1812</v>
@@ -16667,7 +16683,7 @@
         <v>27</v>
       </c>
       <c r="H166" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I166" t="s">
         <v>1819</v>
@@ -16731,7 +16747,7 @@
         <v>27</v>
       </c>
       <c r="H167" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I167" t="s">
         <v>1828</v>
@@ -16855,7 +16871,7 @@
       </c>
       <c r="G169"/>
       <c r="H169" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I169" t="s">
         <v>1847</v>
@@ -16882,7 +16898,7 @@
         <v>1853</v>
       </c>
       <c r="Q169" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R169" t="s">
         <v>1854</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-10-31
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -8993,9 +8993,7 @@
         <v>570</v>
       </c>
       <c r="D47"/>
-      <c r="E47" t="s">
-        <v>168</v>
-      </c>
+      <c r="E47"/>
       <c r="F47" t="s">
         <v>571</v>
       </c>
@@ -13075,9 +13073,7 @@
         <v>570</v>
       </c>
       <c r="D110"/>
-      <c r="E110" t="s">
-        <v>168</v>
-      </c>
+      <c r="E110"/>
       <c r="F110" t="s">
         <v>1263</v>
       </c>
@@ -15021,9 +15017,7 @@
         <v>570</v>
       </c>
       <c r="D140"/>
-      <c r="E140" t="s">
-        <v>168</v>
-      </c>
+      <c r="E140"/>
       <c r="F140" t="s">
         <v>1557</v>
       </c>

</xml_diff>